<commit_message>
upd and pochinka 22
</commit_message>
<xml_diff>
--- a/kompege/zadachi_po_nomeru/task22/20966.xlsx
+++ b/kompege/zadachi_po_nomeru/task22/20966.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elp\Documents\MyGithub\kompege\zadachi_po_nomeru\task22\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\EGEINF\kompege\zadachi_po_nomeru\task22\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BA61DF-007C-41E5-82D3-CACB17F7732C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80E8935-8CC7-4661-BD44-038D8C536467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{A3B4FC9C-C112-49B7-A35F-111DCF2266A0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3B4FC9C-C112-49B7-A35F-111DCF2266A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -574,17 +574,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BA4CF-04E1-42E5-A707-76CD6CB2E487}">
   <dimension ref="A1:AD16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.84375" customWidth="1"/>
-    <col min="3" max="3" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="29" width="3.15234375" customWidth="1"/>
-    <col min="30" max="30" width="3.15234375" style="21" customWidth="1"/>
-    <col min="31" max="70" width="3.15234375" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="29" width="3.109375" customWidth="1"/>
+    <col min="30" max="30" width="3.109375" style="21" customWidth="1"/>
+    <col min="31" max="70" width="3.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +673,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>101</v>
       </c>
@@ -691,7 +691,7 @@
       <c r="I2" s="23"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>102</v>
       </c>
@@ -708,7 +708,7 @@
       <c r="O3" s="23"/>
       <c r="P3" s="8"/>
     </row>
-    <row r="4" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>103</v>
       </c>
@@ -725,7 +725,7 @@
       <c r="X4" s="3"/>
       <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>104</v>
       </c>
@@ -743,7 +743,7 @@
       <c r="V5" s="25"/>
       <c r="W5" s="26"/>
     </row>
-    <row r="6" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>105</v>
       </c>
@@ -760,7 +760,7 @@
       <c r="AB6" s="23"/>
       <c r="AC6" s="23"/>
     </row>
-    <row r="7" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>106</v>
       </c>
@@ -781,7 +781,7 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="14"/>
     </row>
-    <row r="8" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>107</v>
       </c>
@@ -799,7 +799,7 @@
       <c r="O8" s="3"/>
       <c r="P8" s="12"/>
     </row>
-    <row r="9" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>108</v>
       </c>
@@ -812,7 +812,7 @@
       <c r="X9" s="10"/>
       <c r="Y9" s="12"/>
     </row>
-    <row r="10" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>109</v>
       </c>
@@ -825,12 +825,9 @@
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="16"/>
-    </row>
-    <row r="11" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>110</v>
       </c>
@@ -849,7 +846,7 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="19"/>
     </row>
-    <row r="12" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111</v>
       </c>
@@ -862,7 +859,7 @@
       <c r="AA12" s="15"/>
       <c r="AB12" s="4"/>
     </row>
-    <row r="13" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>112</v>
       </c>
@@ -882,7 +879,7 @@
       <c r="Z13" s="3"/>
       <c r="AA13" s="4"/>
     </row>
-    <row r="14" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>113</v>
       </c>
@@ -895,7 +892,7 @@
       <c r="AA14" s="20"/>
       <c r="AB14" s="4"/>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="X16" s="27"/>
       <c r="Y16" s="27"/>
     </row>

</xml_diff>